<commit_message>
Cargue probado y funcionando
</commit_message>
<xml_diff>
--- a/info-cargue-masivo.xlsx
+++ b/info-cargue-masivo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javiz\Documents\Estudio\UT\Semestre 5\Profundización de POO 2\tutoría4\repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C87BBFF2-81FB-4D3D-ABF1-E33F290BA9D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5514D118-38A2-4165-885C-BF77690A1F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E6092881-2855-492E-9194-F35C015A1DE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
   <si>
     <t>PERSONA_ID</t>
   </si>
@@ -59,40 +59,37 @@
     <t>RUTA001</t>
   </si>
   <si>
-    <t>Centro Comercial Multicentro, Ibagué</t>
-  </si>
-  <si>
-    <t>Universidad del Tolima, Ibagué</t>
-  </si>
-  <si>
-    <t>Parque Murillo Toro, Ibagué</t>
-  </si>
-  <si>
     <t>RUTA002</t>
   </si>
   <si>
-    <t>Plaza de Bolívar, Ibagué</t>
-  </si>
-  <si>
-    <t>Clínica Tolima, Ibagué</t>
-  </si>
-  <si>
-    <t>RUTA003</t>
-  </si>
-  <si>
-    <t>SENA Regional Tolima, Ibagué</t>
-  </si>
-  <si>
-    <t>Mercacentro No. 10, Ibagué</t>
-  </si>
-  <si>
-    <t>Estadio Manuel Murillo Toro, Ibagué</t>
-  </si>
-  <si>
-    <t>Aeropuerto Perales, Ibagué</t>
-  </si>
-  <si>
-    <t>Terminal de Transportes, Ibagué</t>
+    <t>Centro Comercial Multicentro Ibagué</t>
+  </si>
+  <si>
+    <t>Universidad del Tolima</t>
+  </si>
+  <si>
+    <t>Parque Murillo Toro</t>
+  </si>
+  <si>
+    <t>Centro Comercial La Estación</t>
+  </si>
+  <si>
+    <t>Plaza de Bolívar Ibagué</t>
+  </si>
+  <si>
+    <t>Terminal de Transporte de Ibagué</t>
+  </si>
+  <si>
+    <t>Clínica Tolima</t>
+  </si>
+  <si>
+    <t>Centro Comercial Acqua</t>
+  </si>
+  <si>
+    <t>Estadio Manuel Murillo Toro</t>
+  </si>
+  <si>
+    <t>Parque Centenario</t>
   </si>
 </sst>
 </file>
@@ -520,13 +517,13 @@
         <v>4</v>
       </c>
       <c r="B2" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1">
         <v>1</v>
@@ -537,13 +534,13 @@
         <v>4</v>
       </c>
       <c r="B3" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" s="1">
         <v>2</v>
@@ -554,13 +551,13 @@
         <v>4</v>
       </c>
       <c r="B4" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4" s="1">
         <v>3</v>
@@ -571,13 +568,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E5" s="1">
         <v>4</v>
@@ -585,104 +582,104 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E6" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B8" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B9" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E9" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B10" s="1">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E10" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B11" s="1">
+        <v>9</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="1">
         <v>5</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="1">
-        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>